<commit_message>
feat(lin): add runtime slave controls and queue-drain receive API
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(lin): document implemented workflows and close roadmap steps 11-12
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
release: bump minor to 0.8.0 and finalize accessibility navigation updates
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -663,6 +663,21 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Evaluate and implement migration from python-can transport to direct Vector XL API (DLL) backend for legacy VectorLINBus adapter while preserving simulation fallback and callback behavior; remove python-can dependency after parity and test migration are complete.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>